<commit_message>
Update company discovery data
</commit_message>
<xml_diff>
--- a/data/company_master_normalized.xlsx
+++ b/data/company_master_normalized.xlsx
@@ -18,16 +18,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -38,7 +35,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -46,21 +43,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -430,167 +418,167 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Company Name</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Normalized Company Name</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Priority</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Industry Focus</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Target Role Family</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Target Keywords</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Major Locations</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Texas Presence</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>H1B Sponsor Signal</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>H1B Evidence URL</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>Official Careers URL</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>Official Job Search URL</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>ATS Type</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>ATS Company Slug</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>Use Official Scraper</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>Monitoring Status</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>Application Status</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>Sponsorship Fit</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>Cold Target Fit</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>Source</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>Source URLs</t>
         </is>
       </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
-      <c r="X1" s="1" t="inlineStr">
+      <c r="X1" t="inlineStr">
         <is>
           <t>Last Checked At</t>
         </is>
       </c>
-      <c r="Y1" s="1" t="inlineStr">
+      <c r="Y1" t="inlineStr">
         <is>
           <t>Last Updated At</t>
         </is>
       </c>
-      <c r="Z1" s="1" t="inlineStr">
+      <c r="Z1" t="inlineStr">
         <is>
           <t>h1b_score</t>
         </is>
       </c>
-      <c r="AA1" s="1" t="inlineStr">
+      <c r="AA1" t="inlineStr">
         <is>
           <t>job_fit_score</t>
         </is>
       </c>
-      <c r="AB1" s="1" t="inlineStr">
+      <c r="AB1" t="inlineStr">
         <is>
           <t>location_score</t>
         </is>
       </c>
-      <c r="AC1" s="1" t="inlineStr">
+      <c r="AC1" t="inlineStr">
         <is>
           <t>industry_fit_score</t>
         </is>
       </c>
-      <c r="AD1" s="1" t="inlineStr">
+      <c r="AD1" t="inlineStr">
         <is>
           <t>investment_score</t>
         </is>
       </c>
-      <c r="AE1" s="1" t="inlineStr">
+      <c r="AE1" t="inlineStr">
         <is>
           <t>source_confidence_score</t>
         </is>
       </c>
-      <c r="AF1" s="1" t="inlineStr">
+      <c r="AF1" t="inlineStr">
         <is>
           <t>overall_company_score</t>
         </is>
       </c>
-      <c r="AG1" s="1" t="inlineStr">
+      <c r="AG1" t="inlineStr">
         <is>
           <t>Recommended Action</t>
         </is>
@@ -60314,37 +60302,37 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>left_index</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>right_index</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>left_company</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>right_company</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>left_normalized</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>right_normalized</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>similarity</t>
         </is>

</xml_diff>